<commit_message>
chore: refresh SpaceX research library
</commit_message>
<xml_diff>
--- a/00_Index.xlsx
+++ b/00_Index.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$47</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -513,7 +513,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -529,6 +529,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -949,7 +952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="2" min="1" max="1"/>
@@ -1216,7 +1219,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>04_Research\Industry</t>
+          <t>04_Research\Starlink</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1226,18 +1229,18 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Industry Research</t>
+          <t>Starlink Research</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Industry context supporting market size, competitive, and Starlink assumptions.</t>
+          <t>Starlink progress report supporting connectivity operating assumptions, subscriber trends, and network capacity context.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Indexed from repository file scan.</t>
+          <t>Relocated from 04_Research\Industry during 2026-06-25 catalog refresh.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1582,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Indexed from repository file scan.</t>
+          <t>Updated workbook in 2026-06-25 working-tree refresh; retained as third-party valuation benchmark.</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1865,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>07_Model</t>
+          <t>07_Model\Archive</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1872,18 +1875,18 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Model Archive</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Valuation model file or model presentation asset.</t>
+          <t>Archived prior valuation model retained for audit trail and pre-IPO assumptions.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Active working model file.</t>
+          <t>Archived from active 07_Model folder during 2026-06-25 refresh; tracked file modified in archive.</t>
         </is>
       </c>
     </row>
@@ -1925,8 +1928,844 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 $25 Billion Inaugural Bond Issuance.pdf</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>02_Investor_Materials</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>SpaceX</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Investor Materials</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Financing material supporting debt capacity, capital structure, liquidity, and interest expense assumptions.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11 Seeking Alpha - Oppenheimer $190 post-IPO Price Target.pdf</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>04_Research\Company</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Company Research</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Company-level market research supporting post-IPO valuation and share price benchmark assumptions.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-19 Reuters - Space startups seek insurance for orbital AI data centers.pdf</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>04_Research\Datacenters</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Datacenter Research</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>AI and orbital datacenter context relevant to xAI/Grok infrastructure, capex, and adjacent-market assumptions.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-24 Seeking Alpha - SpaceX renting out computing may signal another Colossus data center.pdf</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>04_Research\Datacenters</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Datacenter Research</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Datacenter monetization research relevant to AI compute, infrastructure use, and segment optionality assumptions.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Reuters - Firefly Aerospace expected to secure $110 million US EXIM loan.pdf</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>04_Research\Space</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Space Research</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Space-sector financing and competitor context supporting launch market and industry funding assumptions.</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-13 Quartz - SPCX stock opens at $150, tops $2T market cap.pdf</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Quartz</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Market news supporting post-IPO trading, sentiment, and valuation context.</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-16 Forbes - SpaceX Buys Cursor In Largest Startup Acquisition Ever At $60B.pdf</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>M&amp;A news supporting Cursor acquisition assumptions and AI segment valuation context.</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-21 RS Websols - SpaceX Invests $60 Billion to Acquire AI Coding Firm Cursor.pdf</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>RS Websols</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>M&amp;A news supporting Cursor acquisition assumptions and AI segment valuation context.</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22 Motley Fool - SpaceX's Acquisition of Cursor AI Could Be a Massive Bargain.pdf</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Market commentary supporting Cursor acquisition valuation and strategic rationale assumptions.</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22 Reuters - SpaceX turns to bond market, reports $100.8B cash.pdf</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Financing news supporting liquidity, debt issuance, and capital structure assumptions.</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22 Reuters - SpaceX's first week as a public company sparks market mania.pdf</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Post-IPO market news supporting trading, sentiment, and valuation multiple context.</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22 Reuters - X recovers after outage.pdf</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Adjacent-platform operating news relevant to xAI/X ecosystem risk and market context.</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Axiom - SpaceX to borrow $20 billion.pdf</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Axiom</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Debt financing news supporting leverage, liquidity, and refinancing assumptions.</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Reuters - SpaceX extends slump, AI expense concerns grow.pdf</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Market news supporting AI expense risk, sentiment, and downside scenario assumptions.</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Seeking Alpha - SpaceX is said to draw huge demand for first bond sale.pdf</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Debt market demand news supporting credit appetite, financing capacity, and cost of capital assumptions.</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Seeking Alpha - SpaceX sheds $600B in market value amid debt-funding plans.pdf</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Market reaction news supporting valuation sensitivity to leverage, AI spending, and sentiment shifts.</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23 Yahoo Finance - SpaceX debuts bond sale to raise $20 billion after IPO.pdf</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Financing news supporting post-IPO bond issuance, liquidity, and capital structure assumptions.</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-24 Reuters - SpaceX short interest about 5-7% of float.pdf</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Market structure news supporting float, short-interest, and sentiment assumptions.</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-24 Reuters - SpaceX short selling bets increase.pdf</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>05_News</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Market structure news supporting short-interest, volatility, and sentiment assumptions.</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>SpaceX Valuation Model v26.06.24 working.xlsx</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>07_Model\Archive</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Internal Model</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Model Archive</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Archived working valuation model retained for audit trail and assumption comparison.</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>SpaceX Valuation Model v26.06.25 (Cursor Deal + Bond Issuance Refresh).xlsx</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>07_Model</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Internal Model</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Current valuation model refresh incorporating Cursor deal and bond issuance assumptions.</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>2025-12-31 FY25 Cashflow Sankey Diagram.jpg</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>08_Output</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Internal Output</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>FY25 cashflow exhibit supporting model presentation and investment case output materials.</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Cataloged during 2026-06-25 refresh.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H47"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: use versioned model cover
</commit_message>
<xml_diff>
--- a/00_Index.xlsx
+++ b/00_Index.xlsx
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>model-cover.png</t>
+          <t>model-cover-2026-06-25.png</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Model cover screenshot used by README.</t>
+          <t>Renamed from model-cover.png on 2026-06-25 to force refreshed README image rendering.</t>
         </is>
       </c>
     </row>

</xml_diff>